<commit_message>
Use plain MIN/MAX per shelter block in Summary tab
Replaces the _xlfn.MINIFS/_xlfn.MAXIFS earliest/latest-delivery formulas
with plain MIN/MAX over each shelter's contiguous row block on the
All Shelter Checkouts tab. Shelters are grouped, so each block maps to
exactly one shelter (verified programmatically).

The workbook now uses only Excel-2007-era functions (COUNTA, COUNTIF,
COUNTIFS, MIN, MAX, SUM, SUMIF) and no _xlfn-prefixed names, so it
evaluates identically in Excel, LibreOffice and Sheets.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M283xURfMuoYhc5MGYuXwR
</commit_message>
<xml_diff>
--- a/Shelter_Scheduled_Checkouts_2025-2027.xlsx
+++ b/Shelter_Scheduled_Checkouts_2025-2027.xlsx
@@ -8254,11 +8254,11 @@
         <v/>
       </c>
       <c r="I5" s="19">
-        <f>_xlfn.MINIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A5)</f>
+        <f>MIN('All Shelter Checkouts'!$B$5:$B$36)</f>
         <v/>
       </c>
       <c r="J5" s="19">
-        <f>_xlfn.MAXIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A5)</f>
+        <f>MAX('All Shelter Checkouts'!$B$5:$B$36)</f>
         <v/>
       </c>
       <c r="K5" s="20">
@@ -8302,11 +8302,11 @@
         <v/>
       </c>
       <c r="I6" s="19">
-        <f>_xlfn.MINIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A6)</f>
+        <f>MIN('All Shelter Checkouts'!$B$37:$B$41)</f>
         <v/>
       </c>
       <c r="J6" s="19">
-        <f>_xlfn.MAXIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A6)</f>
+        <f>MAX('All Shelter Checkouts'!$B$37:$B$41)</f>
         <v/>
       </c>
       <c r="K6" s="20">
@@ -8350,11 +8350,11 @@
         <v/>
       </c>
       <c r="I7" s="19">
-        <f>_xlfn.MINIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A7)</f>
+        <f>MIN('All Shelter Checkouts'!$B$42:$B$57)</f>
         <v/>
       </c>
       <c r="J7" s="19">
-        <f>_xlfn.MAXIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A7)</f>
+        <f>MAX('All Shelter Checkouts'!$B$42:$B$57)</f>
         <v/>
       </c>
       <c r="K7" s="20">
@@ -8398,11 +8398,11 @@
         <v/>
       </c>
       <c r="I8" s="19">
-        <f>_xlfn.MINIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A8)</f>
+        <f>MIN('All Shelter Checkouts'!$B$58:$B$66)</f>
         <v/>
       </c>
       <c r="J8" s="19">
-        <f>_xlfn.MAXIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A8)</f>
+        <f>MAX('All Shelter Checkouts'!$B$58:$B$66)</f>
         <v/>
       </c>
       <c r="K8" s="20">
@@ -8446,11 +8446,11 @@
         <v/>
       </c>
       <c r="I9" s="19">
-        <f>_xlfn.MINIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A9)</f>
+        <f>MIN('All Shelter Checkouts'!$B$67:$B$68)</f>
         <v/>
       </c>
       <c r="J9" s="19">
-        <f>_xlfn.MAXIFS('All Shelter Checkouts'!$B$5:$B$68,'All Shelter Checkouts'!$A$5:$A$68,$A9)</f>
+        <f>MAX('All Shelter Checkouts'!$B$67:$B$68)</f>
         <v/>
       </c>
       <c r="K9" s="20">

</xml_diff>